<commit_message>
Redo Cuneo Tav. 10: real double reading, 0 validation flags
Re-run with 01b (Senza/TOTALE block location), pass 1 from OCR (01c),
independent visual pass 2 of the strip crops, disagreements decided by
check_pass.py (both block sum and Tav. 1 sum) or by zoomed re-read.
flags_cuneo.csv is empty; tav10_cuneo.dta rebuilt from the validated data.
See docs/audit_2026-10.md.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011mvLWFfLFbnKm7v6S9L2EZ
</commit_message>
<xml_diff>
--- a/output/tav10_cuneo.xlsx
+++ b/output/tav10_cuneo.xlsx
@@ -909,108 +909,112 @@
         <v>1403.25</v>
       </c>
       <c r="AJ2" t="n">
-        <v>0</v>
+        <v>739</v>
       </c>
       <c r="AK2" t="n">
+        <v>4506.08</v>
+      </c>
+      <c r="AL2" t="n">
+        <v>388</v>
+      </c>
+      <c r="AM2" t="n">
         <v>3338.85</v>
       </c>
-      <c r="AL2" t="n">
+      <c r="AN2" t="n">
         <v>183</v>
       </c>
-      <c r="AM2" t="n">
+      <c r="AO2" t="n">
         <v>2026.2</v>
       </c>
-      <c r="AN2" t="n">
+      <c r="AP2" t="n">
         <v>116</v>
       </c>
-      <c r="AO2" t="inlineStr"/>
-      <c r="AP2" t="n">
+      <c r="AQ2" t="n">
+        <v>1590.48</v>
+      </c>
+      <c r="AR2" t="n">
         <v>99</v>
       </c>
-      <c r="AQ2" t="n">
+      <c r="AS2" t="n">
         <v>1707.43</v>
       </c>
-      <c r="AR2" t="n">
+      <c r="AT2" t="n">
         <v>26</v>
       </c>
-      <c r="AS2" t="n">
+      <c r="AU2" t="n">
         <v>572.01</v>
-      </c>
-      <c r="AT2" t="n">
-        <v>12</v>
-      </c>
-      <c r="AU2" t="n">
-        <v>332.43</v>
       </c>
       <c r="AV2" t="n">
         <v>12</v>
       </c>
       <c r="AW2" t="n">
+        <v>332.43</v>
+      </c>
+      <c r="AX2" t="n">
+        <v>12</v>
+      </c>
+      <c r="AY2" t="n">
         <v>403.57</v>
       </c>
-      <c r="AX2" t="n">
+      <c r="AZ2" t="n">
         <v>3</v>
       </c>
-      <c r="AY2" t="n">
+      <c r="BA2" t="n">
         <v>124.48</v>
-      </c>
-      <c r="AZ2" t="n">
-        <v>2</v>
-      </c>
-      <c r="BA2" t="n">
-        <v>126</v>
       </c>
       <c r="BB2" t="n">
         <v>2</v>
       </c>
       <c r="BC2" t="n">
-        <v>162.83</v>
+        <v>126</v>
       </c>
       <c r="BD2" t="n">
         <v>2</v>
       </c>
       <c r="BE2" t="n">
+        <v>162.83</v>
+      </c>
+      <c r="BF2" t="n">
+        <v>2</v>
+      </c>
+      <c r="BG2" t="n">
         <v>251.6</v>
       </c>
-      <c r="BF2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG2" t="n">
-        <v>0</v>
-      </c>
       <c r="BH2" t="n">
         <v>0</v>
       </c>
       <c r="BI2" t="n">
+        <v>0</v>
+      </c>
+      <c r="BJ2" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK2" t="n">
         <v>205</v>
       </c>
-      <c r="BJ2" t="n">
+      <c r="BL2" t="n">
         <v>8</v>
       </c>
-      <c r="BK2" t="n">
+      <c r="BM2" t="n">
         <v>2923.76</v>
       </c>
-      <c r="BL2" t="n">
+      <c r="BN2" t="n">
         <v>2</v>
       </c>
-      <c r="BM2" t="inlineStr"/>
-      <c r="BN2" t="n">
+      <c r="BO2" t="n">
+        <v>1787.23</v>
+      </c>
+      <c r="BP2" t="n">
         <v>8</v>
       </c>
-      <c r="BO2" t="n">
+      <c r="BQ2" t="n">
         <v>11871.26</v>
       </c>
-      <c r="BP2" t="n">
+      <c r="BR2" t="n">
         <v>4</v>
       </c>
-      <c r="BQ2" t="n">
+      <c r="BS2" t="n">
         <v>12622</v>
-      </c>
-      <c r="BR2" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS2" t="n">
-        <v>0</v>
       </c>
       <c r="BT2" t="n">
         <v>4823</v>
@@ -1075,182 +1079,188 @@
       <c r="L3" t="n">
         <v>11</v>
       </c>
-      <c r="M3" t="inlineStr"/>
+      <c r="M3" t="n">
+        <v>4.15</v>
+      </c>
       <c r="N3" t="n">
         <v>4</v>
       </c>
       <c r="O3" t="n">
-        <v>3.99</v>
+        <v>1.96</v>
       </c>
       <c r="P3" t="n">
         <v>6</v>
       </c>
       <c r="Q3" t="n">
+        <v>3.99</v>
+      </c>
+      <c r="R3" t="n">
+        <v>26</v>
+      </c>
+      <c r="S3" t="n">
         <v>24.43</v>
       </c>
-      <c r="R3" t="n">
+      <c r="T3" t="n">
         <v>50</v>
       </c>
-      <c r="S3" t="n">
+      <c r="U3" t="n">
         <v>62.26</v>
       </c>
-      <c r="T3" t="n">
+      <c r="V3" t="n">
         <v>85</v>
       </c>
-      <c r="U3" t="n">
+      <c r="W3" t="n">
         <v>155.12</v>
       </c>
-      <c r="V3" t="n">
+      <c r="X3" t="n">
         <v>87</v>
       </c>
-      <c r="W3" t="n">
+      <c r="Y3" t="n">
         <v>199.07</v>
       </c>
-      <c r="X3" t="n">
+      <c r="Z3" t="n">
         <v>96</v>
       </c>
-      <c r="Y3" t="n">
+      <c r="AA3" t="n">
         <v>276.34</v>
       </c>
-      <c r="Z3" t="n">
+      <c r="AB3" t="n">
         <v>49</v>
       </c>
-      <c r="AA3" t="n">
+      <c r="AC3" t="n">
         <v>160.27</v>
       </c>
-      <c r="AB3" t="n">
+      <c r="AD3" t="n">
         <v>86</v>
       </c>
-      <c r="AC3" t="n">
+      <c r="AE3" t="n">
         <v>334.43</v>
       </c>
-      <c r="AD3" t="n">
+      <c r="AF3" t="n">
         <v>46</v>
       </c>
-      <c r="AE3" t="n">
+      <c r="AG3" t="n">
         <v>195.59</v>
       </c>
-      <c r="AF3" t="n">
+      <c r="AH3" t="n">
         <v>82</v>
       </c>
-      <c r="AG3" t="n">
+      <c r="AI3" t="n">
         <v>400.91</v>
       </c>
-      <c r="AH3" t="n">
+      <c r="AJ3" t="n">
         <v>232</v>
       </c>
-      <c r="AI3" t="n">
+      <c r="AK3" t="n">
         <v>1451.64</v>
       </c>
-      <c r="AJ3" t="n">
+      <c r="AL3" t="n">
         <v>167</v>
       </c>
-      <c r="AK3" t="n">
-        <v>462.28</v>
-      </c>
-      <c r="AL3" t="n">
+      <c r="AM3" t="n">
+        <v>1462.28</v>
+      </c>
+      <c r="AN3" t="n">
         <v>85</v>
       </c>
-      <c r="AM3" t="n">
+      <c r="AO3" t="n">
         <v>956.22</v>
       </c>
-      <c r="AN3" t="n">
+      <c r="AP3" t="n">
         <v>68</v>
       </c>
-      <c r="AO3" t="n">
+      <c r="AQ3" t="n">
         <v>936.22</v>
       </c>
-      <c r="AP3" t="n">
+      <c r="AR3" t="n">
         <v>98</v>
       </c>
-      <c r="AQ3" t="n">
+      <c r="AS3" t="n">
         <v>1709.73</v>
       </c>
-      <c r="AR3" t="n">
+      <c r="AT3" t="n">
         <v>50</v>
       </c>
-      <c r="AS3" t="n">
+      <c r="AU3" t="n">
         <v>1125.72</v>
       </c>
-      <c r="AT3" t="n">
+      <c r="AV3" t="n">
         <v>26</v>
       </c>
-      <c r="AU3" t="n">
+      <c r="AW3" t="n">
         <v>710.13</v>
       </c>
-      <c r="AV3" t="n">
+      <c r="AX3" t="n">
         <v>32</v>
       </c>
-      <c r="AW3" t="n">
+      <c r="AY3" t="n">
         <v>1075.94</v>
       </c>
-      <c r="AX3" t="n">
+      <c r="AZ3" t="n">
         <v>16</v>
       </c>
-      <c r="AY3" t="n">
+      <c r="BA3" t="n">
         <v>719.04</v>
       </c>
-      <c r="AZ3" t="n">
+      <c r="BB3" t="n">
         <v>11</v>
       </c>
-      <c r="BA3" t="n">
+      <c r="BC3" t="n">
         <v>677.4</v>
-      </c>
-      <c r="BB3" t="n">
-        <v>4</v>
-      </c>
-      <c r="BC3" t="n">
-        <v>329.14</v>
       </c>
       <c r="BD3" t="n">
         <v>4</v>
       </c>
       <c r="BE3" t="n">
+        <v>329.14</v>
+      </c>
+      <c r="BF3" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG3" t="n">
         <v>472.38</v>
       </c>
-      <c r="BF3" t="n">
+      <c r="BH3" t="n">
         <v>2</v>
       </c>
-      <c r="BG3" t="n">
+      <c r="BI3" t="n">
         <v>338</v>
       </c>
-      <c r="BH3" t="n">
+      <c r="BJ3" t="n">
         <v>1</v>
       </c>
-      <c r="BI3" t="n">
+      <c r="BK3" t="n">
         <v>210.16</v>
       </c>
-      <c r="BJ3" t="n">
-        <v>4</v>
-      </c>
-      <c r="BK3" t="inlineStr"/>
       <c r="BL3" t="n">
         <v>4</v>
       </c>
       <c r="BM3" t="n">
+        <v>1355.88</v>
+      </c>
+      <c r="BN3" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO3" t="n">
+        <v>3246</v>
+      </c>
+      <c r="BP3" t="n">
+        <v>7</v>
+      </c>
+      <c r="BQ3" t="n">
         <v>11581.69</v>
       </c>
-      <c r="BN3" t="n">
-        <v>7</v>
-      </c>
-      <c r="BO3" t="n">
+      <c r="BR3" t="n">
+        <v>2</v>
+      </c>
+      <c r="BS3" t="n">
         <v>7779</v>
       </c>
-      <c r="BP3" t="n">
-        <v>2</v>
-      </c>
-      <c r="BQ3" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR3" t="n">
+      <c r="BT3" t="n">
         <v>1447</v>
       </c>
-      <c r="BS3" t="inlineStr"/>
-      <c r="BT3" t="n">
-        <v>0</v>
-      </c>
       <c r="BU3" t="n">
-        <v>0</v>
+        <v>37956.12</v>
       </c>
       <c r="BV3" t="inlineStr">
         <is>
@@ -1451,34 +1461,34 @@
         <v>215.93</v>
       </c>
       <c r="BH4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BI4" t="n">
         <v>164.5</v>
       </c>
       <c r="BJ4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK4" t="n">
         <v>214</v>
       </c>
       <c r="BL4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM4" t="n">
-        <v>0</v>
+        <v>416</v>
       </c>
       <c r="BN4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO4" t="n">
-        <v>0</v>
+        <v>674.11</v>
       </c>
       <c r="BP4" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ4" t="n">
-        <v>0</v>
+        <v>1138</v>
       </c>
       <c r="BR4" t="n">
         <v>0</v>
@@ -1487,7 +1497,7 @@
         <v>0</v>
       </c>
       <c r="BT4" t="n">
-        <v>2995</v>
+        <v>2905</v>
       </c>
       <c r="BU4" t="n">
         <v>22543.28</v>
@@ -1655,13 +1665,13 @@
         <v>444.17</v>
       </c>
       <c r="AV5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AW5" t="n">
-        <v>30</v>
+        <v>80</v>
       </c>
       <c r="AX5" t="n">
-        <v>0</v>
+        <v>3</v>
       </c>
       <c r="AY5" t="n">
         <v>110.89</v>
@@ -1673,19 +1683,19 @@
         <v>179.54</v>
       </c>
       <c r="BB5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BC5" t="n">
         <v>50.71</v>
       </c>
       <c r="BD5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE5" t="n">
         <v>87.08</v>
       </c>
       <c r="BF5" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG5" t="n">
         <v>120.32</v>
@@ -1703,28 +1713,28 @@
         <v>0</v>
       </c>
       <c r="BL5" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="BM5" t="n">
+        <v>1452.13</v>
+      </c>
+      <c r="BN5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BO5" t="n">
         <v>2265.57</v>
       </c>
-      <c r="BN5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO5" t="n">
+      <c r="BP5" t="n">
+        <v>3</v>
+      </c>
+      <c r="BQ5" t="n">
         <v>4572.84</v>
       </c>
-      <c r="BP5" t="n">
-        <v>36</v>
-      </c>
-      <c r="BQ5" t="n">
+      <c r="BR5" t="n">
+        <v>6</v>
+      </c>
+      <c r="BS5" t="n">
         <v>27740.26</v>
-      </c>
-      <c r="BR5" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS5" t="n">
-        <v>0</v>
       </c>
       <c r="BT5" t="n">
         <v>1668</v>
@@ -1771,21 +1781,27 @@
       <c r="F6" t="n">
         <v>4</v>
       </c>
-      <c r="G6" t="inlineStr"/>
+      <c r="G6" t="n">
+        <v>0.32</v>
+      </c>
       <c r="H6" t="n">
         <v>18</v>
       </c>
       <c r="I6" t="n">
-        <v>0</v>
+        <v>2.8</v>
       </c>
       <c r="J6" t="n">
         <v>10</v>
       </c>
-      <c r="K6" t="inlineStr"/>
+      <c r="K6" t="n">
+        <v>2.39</v>
+      </c>
       <c r="L6" t="n">
         <v>20</v>
       </c>
-      <c r="M6" t="inlineStr"/>
+      <c r="M6" t="n">
+        <v>7.59</v>
+      </c>
       <c r="N6" t="n">
         <v>13</v>
       </c>
@@ -1795,7 +1811,9 @@
       <c r="P6" t="n">
         <v>42</v>
       </c>
-      <c r="Q6" t="inlineStr"/>
+      <c r="Q6" t="n">
+        <v>25.87</v>
+      </c>
       <c r="R6" t="n">
         <v>54</v>
       </c>
@@ -1805,88 +1823,110 @@
       <c r="T6" t="n">
         <v>99</v>
       </c>
-      <c r="U6" t="inlineStr"/>
-      <c r="V6" t="inlineStr"/>
-      <c r="W6" t="inlineStr"/>
+      <c r="U6" t="n">
+        <v>122.11</v>
+      </c>
+      <c r="V6" t="n">
+        <v>94</v>
+      </c>
+      <c r="W6" t="n">
+        <v>166.55</v>
+      </c>
       <c r="X6" t="n">
         <v>78</v>
       </c>
-      <c r="Y6" t="inlineStr"/>
-      <c r="Z6" t="inlineStr"/>
-      <c r="AA6" t="inlineStr"/>
+      <c r="Y6" t="n">
+        <v>177.69</v>
+      </c>
+      <c r="Z6" t="n">
+        <v>74</v>
+      </c>
+      <c r="AA6" t="n">
+        <v>203.11</v>
+      </c>
       <c r="AB6" t="n">
         <v>90</v>
       </c>
-      <c r="AC6" t="inlineStr"/>
+      <c r="AC6" t="n">
+        <v>286.81</v>
+      </c>
       <c r="AD6" t="n">
         <v>69</v>
       </c>
-      <c r="AE6" t="inlineStr"/>
+      <c r="AE6" t="n">
+        <v>264.25</v>
+      </c>
       <c r="AF6" t="n">
         <v>31</v>
       </c>
-      <c r="AG6" t="inlineStr"/>
+      <c r="AG6" t="n">
+        <v>131.39</v>
+      </c>
       <c r="AH6" t="n">
         <v>63</v>
       </c>
-      <c r="AI6" t="inlineStr"/>
+      <c r="AI6" t="n">
+        <v>301.6</v>
+      </c>
       <c r="AJ6" t="n">
         <v>142</v>
       </c>
       <c r="AK6" t="n">
-        <v>0</v>
+        <v>860.88</v>
       </c>
       <c r="AL6" t="n">
         <v>88</v>
       </c>
       <c r="AM6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AN6" t="inlineStr"/>
+        <v>760.59</v>
+      </c>
+      <c r="AN6" t="n">
+        <v>64</v>
+      </c>
       <c r="AO6" t="n">
-        <v>0</v>
+        <v>699.46</v>
       </c>
       <c r="AP6" t="n">
+        <v>25</v>
+      </c>
+      <c r="AQ6" t="n">
+        <v>344.75</v>
+      </c>
+      <c r="AR6" t="n">
         <v>74</v>
       </c>
-      <c r="AQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR6" t="n">
+      <c r="AS6" t="n">
+        <v>1249.92</v>
+      </c>
+      <c r="AT6" t="n">
         <v>44</v>
       </c>
-      <c r="AS6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT6" t="n">
+      <c r="AU6" t="n">
+        <v>932.33</v>
+      </c>
+      <c r="AV6" t="n">
         <v>22</v>
       </c>
-      <c r="AU6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AV6" t="n">
+      <c r="AW6" t="n">
+        <v>583.75</v>
+      </c>
+      <c r="AX6" t="n">
         <v>18</v>
       </c>
-      <c r="AW6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX6" t="n">
+      <c r="AY6" t="n">
+        <v>567.8</v>
+      </c>
+      <c r="AZ6" t="n">
         <v>10</v>
       </c>
-      <c r="AY6" t="n">
-        <v>0</v>
-      </c>
-      <c r="AZ6" t="n">
+      <c r="BA6" t="n">
+        <v>434.51</v>
+      </c>
+      <c r="BB6" t="n">
         <v>7</v>
       </c>
-      <c r="BA6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB6" t="n">
-        <v>0</v>
-      </c>
       <c r="BC6" t="n">
-        <v>0</v>
+        <v>390.21</v>
       </c>
       <c r="BD6" t="n">
         <v>0</v>
@@ -1895,10 +1935,10 @@
         <v>0</v>
       </c>
       <c r="BF6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG6" t="n">
-        <v>0</v>
+        <v>118.98</v>
       </c>
       <c r="BH6" t="n">
         <v>0</v>
@@ -1913,34 +1953,34 @@
         <v>0</v>
       </c>
       <c r="BL6" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BM6" t="n">
-        <v>0</v>
+        <v>376.23</v>
       </c>
       <c r="BN6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BO6" t="n">
+        <v>0</v>
+      </c>
+      <c r="BP6" t="n">
         <v>2</v>
       </c>
-      <c r="BO6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP6" t="n">
+      <c r="BQ6" t="n">
+        <v>4057.01</v>
+      </c>
+      <c r="BR6" t="n">
         <v>5</v>
       </c>
-      <c r="BQ6" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR6" t="n">
-        <v>0</v>
-      </c>
       <c r="BS6" t="n">
-        <v>0</v>
+        <v>24121.07</v>
       </c>
       <c r="BT6" t="n">
         <v>1268</v>
       </c>
       <c r="BU6" t="n">
-        <v>0</v>
+        <v>37241.96</v>
       </c>
       <c r="BV6" t="inlineStr">
         <is>
@@ -1982,31 +2022,31 @@
         <v>129</v>
       </c>
       <c r="G7" t="n">
-        <v>0</v>
+        <v>9.970000000000001</v>
       </c>
       <c r="H7" t="n">
         <v>195</v>
       </c>
       <c r="I7" t="n">
-        <v>0</v>
+        <v>33.61</v>
       </c>
       <c r="J7" t="n">
         <v>131</v>
       </c>
       <c r="K7" t="n">
-        <v>0</v>
+        <v>34.96</v>
       </c>
       <c r="L7" t="n">
         <v>196</v>
       </c>
       <c r="M7" t="n">
-        <v>0</v>
+        <v>73.38</v>
       </c>
       <c r="N7" t="n">
         <v>97</v>
       </c>
       <c r="O7" t="n">
-        <v>0</v>
+        <v>45.09</v>
       </c>
       <c r="P7" t="n">
         <v>233</v>
@@ -2018,117 +2058,127 @@
         <v>405</v>
       </c>
       <c r="S7" t="n">
-        <v>342.91</v>
+        <v>342.97</v>
       </c>
       <c r="T7" t="n">
         <v>540</v>
       </c>
-      <c r="U7" t="inlineStr"/>
+      <c r="U7" t="n">
+        <v>667.1799999999999</v>
+      </c>
       <c r="V7" t="n">
-        <v>68</v>
+        <v>685</v>
       </c>
       <c r="W7" t="n">
-        <v>0</v>
+        <v>1195.53</v>
       </c>
       <c r="X7" t="n">
+        <v>481</v>
+      </c>
+      <c r="Y7" t="n">
+        <v>1095.6</v>
+      </c>
+      <c r="Z7" t="n">
         <v>461</v>
       </c>
-      <c r="Y7" t="inlineStr"/>
-      <c r="Z7" t="n">
+      <c r="AA7" t="n">
+        <v>1268.46</v>
+      </c>
+      <c r="AB7" t="n">
         <v>462</v>
       </c>
-      <c r="AA7" t="inlineStr"/>
-      <c r="AB7" t="n">
+      <c r="AC7" t="n">
+        <v>1498.69</v>
+      </c>
+      <c r="AD7" t="n">
         <v>397</v>
       </c>
-      <c r="AC7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AD7" t="n">
+      <c r="AE7" t="n">
+        <v>1501.28</v>
+      </c>
+      <c r="AF7" t="n">
         <v>256</v>
       </c>
-      <c r="AE7" t="inlineStr"/>
-      <c r="AF7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AG7" t="inlineStr"/>
+      <c r="AG7" t="n">
+        <v>1088.29</v>
+      </c>
       <c r="AH7" t="n">
-        <v>0</v>
+        <v>358</v>
       </c>
       <c r="AI7" t="n">
+        <v>1696.9</v>
+      </c>
+      <c r="AJ7" t="n">
+        <v>731</v>
+      </c>
+      <c r="AK7" t="n">
         <v>4441.08</v>
       </c>
-      <c r="AJ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AK7" t="n">
-        <v>0</v>
-      </c>
       <c r="AL7" t="n">
-        <v>0</v>
+        <v>346</v>
       </c>
       <c r="AM7" t="n">
-        <v>0</v>
+        <v>2957.92</v>
       </c>
       <c r="AN7" t="n">
-        <v>0</v>
+        <v>113</v>
       </c>
       <c r="AO7" t="n">
-        <v>0</v>
+        <v>1268.09</v>
       </c>
       <c r="AP7" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="AQ7" t="n">
-        <v>0</v>
+        <v>1009.35</v>
       </c>
       <c r="AR7" t="n">
-        <v>0</v>
+        <v>63</v>
       </c>
       <c r="AS7" t="n">
-        <v>0</v>
+        <v>1079.8</v>
       </c>
       <c r="AT7" t="n">
-        <v>0</v>
+        <v>25</v>
       </c>
       <c r="AU7" t="n">
-        <v>0</v>
+        <v>562.58</v>
       </c>
       <c r="AV7" t="n">
+        <v>7</v>
+      </c>
+      <c r="AW7" t="n">
+        <v>195.9</v>
+      </c>
+      <c r="AX7" t="n">
         <v>4</v>
       </c>
-      <c r="AW7" t="n">
-        <v>0</v>
-      </c>
-      <c r="AX7" t="n">
-        <v>0</v>
-      </c>
       <c r="AY7" t="n">
-        <v>0</v>
+        <v>136.49</v>
       </c>
       <c r="AZ7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BA7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BB7" t="n">
         <v>3</v>
       </c>
-      <c r="BA7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BB7" t="n">
-        <v>0</v>
-      </c>
       <c r="BC7" t="n">
-        <v>0</v>
+        <v>169.73</v>
       </c>
       <c r="BD7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BE7" t="n">
+        <v>0</v>
+      </c>
+      <c r="BF7" t="n">
         <v>3</v>
       </c>
-      <c r="BE7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BF7" t="n">
-        <v>0</v>
-      </c>
       <c r="BG7" t="n">
-        <v>0</v>
+        <v>376.05</v>
       </c>
       <c r="BH7" t="n">
         <v>0</v>
@@ -2137,40 +2187,40 @@
         <v>0</v>
       </c>
       <c r="BJ7" t="n">
-        <v>4</v>
+        <v>1</v>
       </c>
       <c r="BK7" t="n">
-        <v>0</v>
+        <v>222.56</v>
       </c>
       <c r="BL7" t="n">
         <v>4</v>
       </c>
       <c r="BM7" t="n">
-        <v>0</v>
+        <v>1453.17</v>
       </c>
       <c r="BN7" t="n">
+        <v>4</v>
+      </c>
+      <c r="BO7" t="n">
+        <v>3191.63</v>
+      </c>
+      <c r="BP7" t="n">
         <v>2</v>
       </c>
-      <c r="BO7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BP7" t="n">
+      <c r="BQ7" t="n">
+        <v>2510.01</v>
+      </c>
+      <c r="BR7" t="n">
         <v>1</v>
       </c>
-      <c r="BQ7" t="n">
-        <v>0</v>
-      </c>
-      <c r="BR7" t="n">
-        <v>0</v>
-      </c>
       <c r="BS7" t="n">
-        <v>0</v>
+        <v>3466.35</v>
       </c>
       <c r="BT7" t="n">
-        <v>8418</v>
+        <v>6416</v>
       </c>
       <c r="BU7" t="n">
-        <v>0</v>
+        <v>33735.21</v>
       </c>
       <c r="BV7" t="inlineStr">
         <is>
@@ -2356,55 +2406,55 @@
         <v>5</v>
       </c>
       <c r="BC8" t="n">
-        <v>0</v>
+        <v>299.19</v>
       </c>
       <c r="BD8" t="n">
         <v>4</v>
       </c>
       <c r="BE8" t="n">
+        <v>362.6</v>
+      </c>
+      <c r="BF8" t="n">
+        <v>4</v>
+      </c>
+      <c r="BG8" t="n">
         <v>531.4299999999999</v>
       </c>
-      <c r="BF8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG8" t="n">
+      <c r="BH8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI8" t="n">
         <v>152.81</v>
       </c>
-      <c r="BH8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI8" t="n">
+      <c r="BJ8" t="n">
+        <v>3</v>
+      </c>
+      <c r="BK8" t="n">
         <v>655.09</v>
       </c>
-      <c r="BJ8" t="n">
+      <c r="BL8" t="n">
         <v>10</v>
       </c>
-      <c r="BK8" t="n">
+      <c r="BM8" t="n">
         <v>3957.64</v>
       </c>
-      <c r="BL8" t="n">
+      <c r="BN8" t="n">
         <v>5</v>
       </c>
-      <c r="BM8" t="n">
+      <c r="BO8" t="n">
         <v>4048.6</v>
       </c>
-      <c r="BN8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO8" t="n">
+      <c r="BP8" t="n">
+        <v>5</v>
+      </c>
+      <c r="BQ8" t="n">
         <v>7378.42</v>
       </c>
-      <c r="BP8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ8" t="n">
+      <c r="BR8" t="n">
+        <v>1</v>
+      </c>
+      <c r="BS8" t="n">
         <v>4745</v>
-      </c>
-      <c r="BR8" t="n">
-        <v>0</v>
-      </c>
-      <c r="BS8" t="n">
-        <v>0</v>
       </c>
       <c r="BT8" t="n">
         <v>4264</v>
@@ -2505,7 +2555,9 @@
       <c r="X9" t="n">
         <v>116</v>
       </c>
-      <c r="Y9" t="inlineStr"/>
+      <c r="Y9" t="n">
+        <v>266.98</v>
+      </c>
       <c r="Z9" t="n">
         <v>130</v>
       </c>
@@ -2545,7 +2597,9 @@
       <c r="AL9" t="n">
         <v>308</v>
       </c>
-      <c r="AM9" t="inlineStr"/>
+      <c r="AM9" t="n">
+        <v>2687.61</v>
+      </c>
       <c r="AN9" t="n">
         <v>168</v>
       </c>
@@ -2580,61 +2634,61 @@
         <v>40</v>
       </c>
       <c r="AY9" t="n">
-        <v>628.97</v>
+        <v>1325.15</v>
       </c>
       <c r="AZ9" t="n">
         <v>14</v>
       </c>
       <c r="BA9" t="n">
-        <v>488.13</v>
+        <v>628.97</v>
       </c>
       <c r="BB9" t="n">
         <v>8</v>
       </c>
       <c r="BC9" t="n">
+        <v>488.13</v>
+      </c>
+      <c r="BD9" t="n">
+        <v>4</v>
+      </c>
+      <c r="BE9" t="n">
         <v>338.81</v>
       </c>
-      <c r="BD9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BE9" t="n">
+      <c r="BF9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BG9" t="n">
         <v>107.5</v>
       </c>
-      <c r="BF9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BG9" t="n">
+      <c r="BH9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BI9" t="n">
         <v>177.87</v>
       </c>
-      <c r="BH9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI9" t="n">
+      <c r="BJ9" t="n">
+        <v>1</v>
+      </c>
+      <c r="BK9" t="n">
         <v>219.13</v>
       </c>
-      <c r="BJ9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BK9" t="n">
-        <v>0</v>
-      </c>
       <c r="BL9" t="n">
-        <v>2</v>
+        <v>0</v>
       </c>
       <c r="BM9" t="n">
-        <v>1140.05</v>
+        <v>0</v>
       </c>
       <c r="BN9" t="n">
         <v>2</v>
       </c>
       <c r="BO9" t="n">
+        <v>1140.05</v>
+      </c>
+      <c r="BP9" t="n">
+        <v>2</v>
+      </c>
+      <c r="BQ9" t="n">
         <v>3611</v>
-      </c>
-      <c r="BP9" t="n">
-        <v>0</v>
-      </c>
-      <c r="BQ9" t="n">
-        <v>0</v>
       </c>
       <c r="BR9" t="n">
         <v>0</v>
@@ -2796,7 +2850,7 @@
         <v>73</v>
       </c>
       <c r="AQ10" t="n">
-        <v>8.369999999999999</v>
+        <v>1008.37</v>
       </c>
       <c r="AR10" t="n">
         <v>87</v>
@@ -2813,11 +2867,15 @@
       <c r="AV10" t="n">
         <v>12</v>
       </c>
-      <c r="AW10" t="inlineStr"/>
+      <c r="AW10" t="n">
+        <v>325.02</v>
+      </c>
       <c r="AX10" t="n">
         <v>23</v>
       </c>
-      <c r="AY10" t="inlineStr"/>
+      <c r="AY10" t="n">
+        <v>796.6</v>
+      </c>
       <c r="AZ10" t="n">
         <v>7</v>
       </c>
@@ -2861,16 +2919,16 @@
         <v>0</v>
       </c>
       <c r="BN10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BO10" t="n">
-        <v>0</v>
+        <v>699.03</v>
       </c>
       <c r="BP10" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BQ10" t="n">
-        <v>0</v>
+        <v>2108</v>
       </c>
       <c r="BR10" t="n">
         <v>0</v>
@@ -2881,7 +2939,9 @@
       <c r="BT10" t="n">
         <v>5497</v>
       </c>
-      <c r="BU10" t="inlineStr"/>
+      <c r="BU10" t="n">
+        <v>24598.36</v>
+      </c>
       <c r="BV10" t="inlineStr">
         <is>
           <t>C</t>
@@ -2922,7 +2982,7 @@
         <v>80</v>
       </c>
       <c r="G11" t="n">
-        <v>0</v>
+        <v>6.75</v>
       </c>
       <c r="H11" t="n">
         <v>287</v>
@@ -2939,7 +2999,9 @@
       <c r="L11" t="n">
         <v>346</v>
       </c>
-      <c r="M11" t="inlineStr"/>
+      <c r="M11" t="n">
+        <v>128.83</v>
+      </c>
       <c r="N11" t="n">
         <v>177</v>
       </c>
@@ -2961,7 +3023,9 @@
       <c r="T11" t="n">
         <v>865</v>
       </c>
-      <c r="U11" t="inlineStr"/>
+      <c r="U11" t="n">
+        <v>1082.63</v>
+      </c>
       <c r="V11" t="n">
         <v>1035</v>
       </c>
@@ -2971,7 +3035,9 @@
       <c r="X11" t="n">
         <v>846</v>
       </c>
-      <c r="Y11" t="inlineStr"/>
+      <c r="Y11" t="n">
+        <v>1923.57</v>
+      </c>
       <c r="Z11" t="n">
         <v>692</v>
       </c>
@@ -3042,25 +3108,25 @@
         <v>23</v>
       </c>
       <c r="AW11" t="n">
-        <v>0</v>
+        <v>628.39</v>
       </c>
       <c r="AX11" t="n">
         <v>36</v>
       </c>
       <c r="AY11" t="n">
-        <v>0</v>
+        <v>1224.39</v>
       </c>
       <c r="AZ11" t="n">
         <v>15</v>
       </c>
       <c r="BA11" t="n">
-        <v>0</v>
+        <v>661.5</v>
       </c>
       <c r="BB11" t="n">
         <v>7</v>
       </c>
       <c r="BC11" t="n">
-        <v>0</v>
+        <v>404.02</v>
       </c>
       <c r="BD11" t="n">
         <v>0</v>
@@ -3069,10 +3135,10 @@
         <v>0</v>
       </c>
       <c r="BF11" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BG11" t="n">
-        <v>0</v>
+        <v>104.49</v>
       </c>
       <c r="BH11" t="n">
         <v>0</v>
@@ -3114,7 +3180,7 @@
         <v>9185</v>
       </c>
       <c r="BU11" t="n">
-        <v>0</v>
+        <v>32565.45</v>
       </c>
       <c r="BV11" t="inlineStr">
         <is>
@@ -3153,22 +3219,22 @@
         <v>0</v>
       </c>
       <c r="F12" t="n">
-        <v>0</v>
+        <v>42</v>
       </c>
       <c r="G12" t="n">
-        <v>0</v>
+        <v>2.99</v>
       </c>
       <c r="H12" t="n">
-        <v>42</v>
+        <v>143</v>
       </c>
       <c r="I12" t="n">
-        <v>2.99</v>
+        <v>23.76</v>
       </c>
       <c r="J12" t="n">
-        <v>143</v>
+        <v>120</v>
       </c>
       <c r="K12" t="n">
-        <v>23.76</v>
+        <v>31.12</v>
       </c>
       <c r="L12" t="n">
         <v>188</v>
@@ -3351,10 +3417,10 @@
         <v>0</v>
       </c>
       <c r="BT12" t="n">
-        <v>0</v>
+        <v>7382</v>
       </c>
       <c r="BU12" t="n">
-        <v>0</v>
+        <v>29772.93</v>
       </c>
       <c r="BV12" t="inlineStr">
         <is>
@@ -3393,37 +3459,37 @@
         <v>0</v>
       </c>
       <c r="F13" t="n">
-        <v>0</v>
+        <v>4</v>
       </c>
       <c r="G13" t="n">
-        <v>0</v>
+        <v>0.26</v>
       </c>
       <c r="H13" t="n">
-        <v>4</v>
+        <v>26</v>
       </c>
       <c r="I13" t="n">
-        <v>0.26</v>
+        <v>4.72</v>
       </c>
       <c r="J13" t="n">
-        <v>26</v>
+        <v>13</v>
       </c>
       <c r="K13" t="n">
-        <v>0</v>
+        <v>3.4</v>
       </c>
       <c r="L13" t="n">
-        <v>13</v>
+        <v>55</v>
       </c>
       <c r="M13" t="n">
-        <v>0</v>
+        <v>20.62</v>
       </c>
       <c r="N13" t="n">
-        <v>0</v>
+        <v>14</v>
       </c>
       <c r="O13" t="n">
         <v>6.37</v>
       </c>
       <c r="P13" t="n">
-        <v>0</v>
+        <v>55</v>
       </c>
       <c r="Q13" t="n">
         <v>32.9</v>
@@ -3501,7 +3567,7 @@
         <v>3578.58</v>
       </c>
       <c r="AP13" t="n">
-        <v>175</v>
+        <v>178</v>
       </c>
       <c r="AQ13" t="n">
         <v>2434.1</v>
@@ -3591,10 +3657,10 @@
         <v>0</v>
       </c>
       <c r="BT13" t="n">
-        <v>0</v>
+        <v>3944</v>
       </c>
       <c r="BU13" t="n">
-        <v>0</v>
+        <v>26025.24</v>
       </c>
       <c r="BV13" t="inlineStr">
         <is>
@@ -3633,144 +3699,148 @@
         <v>0</v>
       </c>
       <c r="F14" t="n">
-        <v>0</v>
+        <v>16</v>
       </c>
       <c r="G14" t="n">
-        <v>0</v>
+        <v>1.3</v>
       </c>
       <c r="H14" t="n">
-        <v>0</v>
+        <v>52</v>
       </c>
       <c r="I14" t="n">
-        <v>0</v>
+        <v>8.859999999999999</v>
       </c>
       <c r="J14" t="n">
-        <v>0</v>
+        <v>47</v>
       </c>
       <c r="K14" t="n">
-        <v>0</v>
+        <v>12.11</v>
       </c>
       <c r="L14" t="n">
-        <v>0</v>
+        <v>74</v>
       </c>
       <c r="M14" t="n">
-        <v>0</v>
+        <v>27.84</v>
       </c>
       <c r="N14" t="n">
-        <v>0</v>
+        <v>51</v>
       </c>
       <c r="O14" t="n">
-        <v>0</v>
+        <v>23.57</v>
       </c>
       <c r="P14" t="n">
-        <v>0</v>
+        <v>95</v>
       </c>
       <c r="Q14" t="n">
-        <v>0</v>
+        <v>58.48</v>
       </c>
       <c r="R14" t="n">
-        <v>0</v>
+        <v>166</v>
       </c>
       <c r="S14" t="n">
-        <v>0</v>
+        <v>142.12</v>
       </c>
       <c r="T14" t="n">
-        <v>0</v>
+        <v>241</v>
       </c>
       <c r="U14" t="n">
-        <v>0</v>
+        <v>305.96</v>
       </c>
       <c r="V14" t="n">
-        <v>0</v>
+        <v>350</v>
       </c>
       <c r="W14" t="n">
-        <v>0</v>
+        <v>614.67</v>
       </c>
       <c r="X14" t="n">
-        <v>0</v>
+        <v>255</v>
       </c>
       <c r="Y14" t="n">
-        <v>0</v>
+        <v>584.0700000000001</v>
       </c>
       <c r="Z14" t="n">
-        <v>0</v>
+        <v>257</v>
       </c>
       <c r="AA14" t="n">
-        <v>0</v>
+        <v>706.72</v>
       </c>
       <c r="AB14" t="n">
-        <v>0</v>
+        <v>359</v>
       </c>
       <c r="AC14" t="n">
-        <v>0</v>
+        <v>1165.6</v>
       </c>
       <c r="AD14" t="n">
-        <v>0</v>
+        <v>232</v>
       </c>
       <c r="AE14" t="n">
-        <v>0</v>
+        <v>880.84</v>
       </c>
       <c r="AF14" t="n">
-        <v>0</v>
+        <v>172</v>
       </c>
       <c r="AG14" t="n">
-        <v>0</v>
+        <v>730.72</v>
       </c>
       <c r="AH14" t="n">
         <v>287</v>
       </c>
       <c r="AI14" t="n">
-        <v>0</v>
+        <v>1365.02</v>
       </c>
       <c r="AJ14" t="n">
         <v>843</v>
       </c>
       <c r="AK14" t="n">
-        <v>0</v>
+        <v>5195.07</v>
       </c>
       <c r="AL14" t="n">
         <v>581</v>
       </c>
       <c r="AM14" t="n">
-        <v>0</v>
+        <v>4999.81</v>
       </c>
       <c r="AN14" t="n">
         <v>246</v>
       </c>
       <c r="AO14" t="n">
-        <v>0</v>
+        <v>2734.97</v>
       </c>
       <c r="AP14" t="n">
-        <v>54</v>
+        <v>154</v>
       </c>
       <c r="AQ14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AR14" t="inlineStr"/>
+        <v>2096.6</v>
+      </c>
+      <c r="AR14" t="n">
+        <v>152</v>
+      </c>
       <c r="AS14" t="n">
-        <v>0</v>
-      </c>
-      <c r="AT14" t="inlineStr"/>
+        <v>2616.98</v>
+      </c>
+      <c r="AT14" t="n">
+        <v>43</v>
+      </c>
       <c r="AU14" t="n">
-        <v>0</v>
+        <v>948.53</v>
       </c>
       <c r="AV14" t="n">
         <v>19</v>
       </c>
       <c r="AW14" t="n">
-        <v>0</v>
+        <v>513.35</v>
       </c>
       <c r="AX14" t="n">
-        <v>0</v>
+        <v>10</v>
       </c>
       <c r="AY14" t="n">
-        <v>0</v>
+        <v>334.84</v>
       </c>
       <c r="AZ14" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BA14" t="n">
-        <v>0</v>
+        <v>215.07</v>
       </c>
       <c r="BB14" t="n">
         <v>0</v>
@@ -3779,10 +3849,10 @@
         <v>0</v>
       </c>
       <c r="BD14" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE14" t="n">
-        <v>0</v>
+        <v>80</v>
       </c>
       <c r="BF14" t="n">
         <v>0</v>
@@ -3827,10 +3897,10 @@
         <v>0</v>
       </c>
       <c r="BT14" t="n">
-        <v>8</v>
+        <v>4708</v>
       </c>
       <c r="BU14" t="n">
-        <v>0</v>
+        <v>26363.1</v>
       </c>
       <c r="BV14" t="inlineStr">
         <is>
@@ -3872,145 +3942,145 @@
         <v>24</v>
       </c>
       <c r="G15" t="n">
-        <v>0</v>
+        <v>2.06</v>
       </c>
       <c r="H15" t="n">
         <v>78</v>
       </c>
       <c r="I15" t="n">
-        <v>0</v>
+        <v>13.88</v>
       </c>
       <c r="J15" t="n">
         <v>43</v>
       </c>
       <c r="K15" t="n">
-        <v>0</v>
+        <v>11.52</v>
       </c>
       <c r="L15" t="n">
         <v>144</v>
       </c>
       <c r="M15" t="n">
-        <v>0</v>
+        <v>54.41</v>
       </c>
       <c r="N15" t="n">
         <v>47</v>
       </c>
       <c r="O15" t="n">
-        <v>0</v>
+        <v>21.85</v>
       </c>
       <c r="P15" t="n">
         <v>137</v>
       </c>
       <c r="Q15" t="n">
-        <v>0</v>
+        <v>80.84</v>
       </c>
       <c r="R15" t="n">
         <v>280</v>
       </c>
       <c r="S15" t="n">
-        <v>0</v>
+        <v>235.62</v>
       </c>
       <c r="T15" t="n">
-        <v>0</v>
+        <v>314</v>
       </c>
       <c r="U15" t="n">
-        <v>0</v>
+        <v>380.17</v>
       </c>
       <c r="V15" t="n">
-        <v>0</v>
+        <v>463</v>
       </c>
       <c r="W15" t="n">
-        <v>0</v>
+        <v>811.17</v>
       </c>
       <c r="X15" t="n">
-        <v>0</v>
+        <v>339</v>
       </c>
       <c r="Y15" t="n">
-        <v>0</v>
+        <v>771.64</v>
       </c>
       <c r="Z15" t="n">
-        <v>0</v>
+        <v>298</v>
       </c>
       <c r="AA15" t="n">
-        <v>0</v>
+        <v>813.76</v>
       </c>
       <c r="AB15" t="n">
-        <v>0</v>
+        <v>424</v>
       </c>
       <c r="AC15" t="n">
-        <v>0</v>
+        <v>1370.9</v>
       </c>
       <c r="AD15" t="n">
-        <v>0</v>
+        <v>333</v>
       </c>
       <c r="AE15" t="n">
-        <v>0</v>
+        <v>1266.16</v>
       </c>
       <c r="AF15" t="n">
-        <v>0</v>
+        <v>243</v>
       </c>
       <c r="AG15" t="n">
-        <v>0</v>
+        <v>1027.65</v>
       </c>
       <c r="AH15" t="n">
-        <v>0</v>
+        <v>364</v>
       </c>
       <c r="AI15" t="n">
-        <v>0</v>
+        <v>1722.87</v>
       </c>
       <c r="AJ15" t="n">
         <v>992</v>
       </c>
       <c r="AK15" t="n">
-        <v>0</v>
+        <v>6122.19</v>
       </c>
       <c r="AL15" t="n">
         <v>514</v>
       </c>
       <c r="AM15" t="n">
-        <v>0</v>
+        <v>4424.82</v>
       </c>
       <c r="AN15" t="n">
         <v>196</v>
       </c>
       <c r="AO15" t="n">
-        <v>0</v>
+        <v>2197.49</v>
       </c>
       <c r="AP15" t="n">
         <v>123</v>
       </c>
       <c r="AQ15" t="n">
-        <v>0</v>
+        <v>1676.8</v>
       </c>
       <c r="AR15" t="n">
         <v>127</v>
       </c>
       <c r="AS15" t="n">
-        <v>0</v>
+        <v>2145.23</v>
       </c>
       <c r="AT15" t="n">
         <v>33</v>
       </c>
       <c r="AU15" t="n">
-        <v>0</v>
+        <v>733.03</v>
       </c>
       <c r="AV15" t="n">
         <v>30</v>
       </c>
       <c r="AW15" t="n">
-        <v>0</v>
+        <v>809.09</v>
       </c>
       <c r="AX15" t="n">
         <v>11</v>
       </c>
       <c r="AY15" t="n">
-        <v>0</v>
+        <v>380.13</v>
       </c>
       <c r="AZ15" t="n">
         <v>2</v>
       </c>
       <c r="BA15" t="n">
-        <v>0</v>
+        <v>81.48999999999999</v>
       </c>
       <c r="BB15" t="n">
         <v>0</v>
@@ -4019,16 +4089,16 @@
         <v>0</v>
       </c>
       <c r="BD15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BE15" t="n">
-        <v>0</v>
+        <v>84.43000000000001</v>
       </c>
       <c r="BF15" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG15" t="n">
-        <v>0</v>
+        <v>248.25</v>
       </c>
       <c r="BH15" t="n">
         <v>0</v>
@@ -4037,10 +4107,10 @@
         <v>0</v>
       </c>
       <c r="BJ15" t="n">
-        <v>0</v>
+        <v>1</v>
       </c>
       <c r="BK15" t="n">
-        <v>0</v>
+        <v>225</v>
       </c>
       <c r="BL15" t="n">
         <v>0</v>
@@ -4052,7 +4122,7 @@
         <v>2</v>
       </c>
       <c r="BO15" t="n">
-        <v>0</v>
+        <v>1413.06</v>
       </c>
       <c r="BP15" t="n">
         <v>0</v>
@@ -4067,10 +4137,10 @@
         <v>0</v>
       </c>
       <c r="BT15" t="n">
-        <v>0</v>
+        <v>5567</v>
       </c>
       <c r="BU15" t="n">
-        <v>0</v>
+        <v>29125.51</v>
       </c>
       <c r="BV15" t="inlineStr">
         <is>
@@ -4195,11 +4265,15 @@
       <c r="AH16" t="n">
         <v>240</v>
       </c>
-      <c r="AI16" t="inlineStr"/>
+      <c r="AI16" t="n">
+        <v>1139.6</v>
+      </c>
       <c r="AJ16" t="n">
         <v>751</v>
       </c>
-      <c r="AK16" t="inlineStr"/>
+      <c r="AK16" t="n">
+        <v>4673.75</v>
+      </c>
       <c r="AL16" t="n">
         <v>607</v>
       </c>
@@ -4237,53 +4311,53 @@
         <v>5330.76</v>
       </c>
       <c r="AX16" t="n">
-        <v>64</v>
+        <v>219</v>
       </c>
       <c r="AY16" t="n">
         <v>7438</v>
       </c>
       <c r="AZ16" t="n">
-        <v>0</v>
+        <v>64</v>
       </c>
       <c r="BA16" t="n">
-        <v>0</v>
+        <v>2828.63</v>
       </c>
       <c r="BB16" t="n">
+        <v>51</v>
+      </c>
+      <c r="BC16" t="n">
+        <v>3046.69</v>
+      </c>
+      <c r="BD16" t="n">
         <v>7</v>
       </c>
-      <c r="BC16" t="n">
+      <c r="BE16" t="n">
         <v>581.11</v>
       </c>
-      <c r="BD16" t="n">
+      <c r="BF16" t="n">
         <v>4</v>
       </c>
-      <c r="BE16" t="n">
+      <c r="BG16" t="n">
         <v>449.61</v>
       </c>
-      <c r="BF16" t="n">
+      <c r="BH16" t="n">
         <v>2</v>
       </c>
-      <c r="BG16" t="n">
+      <c r="BI16" t="n">
         <v>368.15</v>
       </c>
-      <c r="BH16" t="n">
-        <v>0</v>
-      </c>
-      <c r="BI16" t="n">
-        <v>0</v>
-      </c>
       <c r="BJ16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BK16" t="n">
+        <v>0</v>
+      </c>
+      <c r="BL16" t="n">
         <v>2</v>
       </c>
-      <c r="BK16" t="n">
+      <c r="BM16" t="n">
         <v>685.86</v>
       </c>
-      <c r="BL16" t="n">
-        <v>0</v>
-      </c>
-      <c r="BM16" t="n">
-        <v>0</v>
-      </c>
       <c r="BN16" t="n">
         <v>0</v>
       </c>
@@ -4302,7 +4376,9 @@
       <c r="BS16" t="n">
         <v>0</v>
       </c>
-      <c r="BT16" t="inlineStr"/>
+      <c r="BT16" t="n">
+        <v>6314</v>
+      </c>
       <c r="BU16" t="n">
         <v>58388.83</v>
       </c>
@@ -4375,15 +4451,21 @@
       <c r="P17" t="n">
         <v>278</v>
       </c>
-      <c r="Q17" t="inlineStr"/>
+      <c r="Q17" t="n">
+        <v>172.25</v>
+      </c>
       <c r="R17" t="n">
         <v>390</v>
       </c>
-      <c r="S17" t="inlineStr"/>
+      <c r="S17" t="n">
+        <v>329.8</v>
+      </c>
       <c r="T17" t="n">
         <v>414</v>
       </c>
-      <c r="U17" t="inlineStr"/>
+      <c r="U17" t="n">
+        <v>508.98</v>
+      </c>
       <c r="V17" t="n">
         <v>416</v>
       </c>
@@ -4471,7 +4553,9 @@
       <c r="AX17" t="n">
         <v>41</v>
       </c>
-      <c r="AY17" t="inlineStr"/>
+      <c r="AY17" t="n">
+        <v>1417.64</v>
+      </c>
       <c r="AZ17" t="n">
         <v>10</v>
       </c>
@@ -4479,22 +4563,22 @@
         <v>450.08</v>
       </c>
       <c r="BB17" t="n">
-        <v>0</v>
+        <v>5</v>
       </c>
       <c r="BC17" t="n">
         <v>278.72</v>
       </c>
       <c r="BD17" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="BE17" t="n">
         <v>234.14</v>
       </c>
       <c r="BF17" t="n">
-        <v>0</v>
+        <v>2</v>
       </c>
       <c r="BG17" t="n">
-        <v>0</v>
+        <v>265.4</v>
       </c>
       <c r="BH17" t="n">
         <v>0</v>
@@ -4512,13 +4596,13 @@
         <v>0</v>
       </c>
       <c r="BM17" t="n">
+        <v>0</v>
+      </c>
+      <c r="BN17" t="n">
+        <v>1</v>
+      </c>
+      <c r="BO17" t="n">
         <v>927.29</v>
-      </c>
-      <c r="BN17" t="n">
-        <v>0</v>
-      </c>
-      <c r="BO17" t="n">
-        <v>0</v>
       </c>
       <c r="BP17" t="n">
         <v>0</v>
@@ -4655,11 +4739,15 @@
       <c r="AF18" t="n">
         <v>293</v>
       </c>
-      <c r="AG18" t="inlineStr"/>
+      <c r="AG18" t="n">
+        <v>1237.87</v>
+      </c>
       <c r="AH18" t="n">
         <v>478</v>
       </c>
-      <c r="AI18" t="inlineStr"/>
+      <c r="AI18" t="n">
+        <v>2262.76</v>
+      </c>
       <c r="AJ18" t="n">
         <v>1289</v>
       </c>
@@ -4675,7 +4763,9 @@
       <c r="AN18" t="n">
         <v>415</v>
       </c>
-      <c r="AO18" t="inlineStr"/>
+      <c r="AO18" t="n">
+        <v>4658.39</v>
+      </c>
       <c r="AP18" t="n">
         <v>281</v>
       </c>
@@ -4698,31 +4788,31 @@
         <v>69</v>
       </c>
       <c r="AW18" t="n">
-        <v>0</v>
+        <v>1857.73</v>
       </c>
       <c r="AX18" t="n">
         <v>50</v>
       </c>
       <c r="AY18" t="n">
-        <v>0</v>
+        <v>1663.07</v>
       </c>
       <c r="AZ18" t="n">
         <v>8</v>
       </c>
       <c r="BA18" t="n">
-        <v>0</v>
+        <v>352.99</v>
       </c>
       <c r="BB18" t="n">
         <v>8</v>
       </c>
       <c r="BC18" t="n">
-        <v>0</v>
+        <v>473.93</v>
       </c>
       <c r="BD18" t="n">
         <v>5</v>
       </c>
       <c r="BE18" t="n">
-        <v>0</v>
+        <v>427.15</v>
       </c>
       <c r="BF18" t="n">
         <v>4</v>
@@ -4766,9 +4856,11 @@
       <c r="BS18" t="n">
         <v>0</v>
       </c>
-      <c r="BT18" t="inlineStr"/>
+      <c r="BT18" t="n">
+        <v>8086</v>
+      </c>
       <c r="BU18" t="n">
-        <v>0</v>
+        <v>49289.57</v>
       </c>
       <c r="BV18" t="inlineStr">
         <is>

</xml_diff>